<commit_message>
Ganti No Gudang 103 ke 515 pada Blok 06 (Saf 6, Tingkat 3)
</commit_message>
<xml_diff>
--- a/c.xlsx
+++ b/c.xlsx
@@ -3998,16 +3998,16 @@
         </is>
       </c>
       <c r="R73" s="11" t="n">
-        <v>103</v>
+        <v>515</v>
       </c>
       <c r="S73" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32957</t>
         </is>
       </c>
       <c r="T73" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>36.0 kg</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="E87" s="13" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>45.0 kg</t>
         </is>
       </c>
       <c r="F87" s="11" t="n">
@@ -11281,7 +11281,7 @@
         <v>387</v>
       </c>
       <c r="H61" s="14" t="n">
-        <v>103</v>
+        <v>515</v>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
@@ -15470,16 +15470,16 @@
         </is>
       </c>
       <c r="P44" s="18" t="n">
-        <v>103</v>
+        <v>515</v>
       </c>
       <c r="Q44" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32957</t>
         </is>
       </c>
       <c r="R44" s="13" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>36.0 kg</t>
         </is>
       </c>
     </row>
@@ -15957,7 +15957,7 @@
       </c>
       <c r="C53" s="13" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>45.0 kg</t>
         </is>
       </c>
       <c r="D53" s="18" t="n">
@@ -19753,7 +19753,7 @@
         <v>18</v>
       </c>
       <c r="I13" s="25" t="n">
-        <v>830</v>
+        <v>866</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -25906,21 +25906,21 @@
         <v>135</v>
       </c>
       <c r="C163" s="18" t="n">
-        <v>103</v>
+        <v>515</v>
       </c>
       <c r="D163" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>32957</t>
         </is>
       </c>
       <c r="E163" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>66</t>
         </is>
       </c>
       <c r="F163" s="29" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>36.0 kg</t>
         </is>
       </c>
       <c r="G163" s="28" t="inlineStr">
@@ -25940,7 +25940,7 @@
       </c>
       <c r="J163" s="28" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
     </row>
@@ -27253,7 +27253,7 @@
       </c>
       <c r="F194" s="33" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>45.0 kg</t>
         </is>
       </c>
       <c r="G194" s="30" t="inlineStr">

</xml_diff>

<commit_message>
Sync c.xlsx and stock susunan reports with updated Supabase
</commit_message>
<xml_diff>
--- a/c.xlsx
+++ b/c.xlsx
@@ -977,16 +977,16 @@
         </is>
       </c>
       <c r="L11" s="11" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>35080</t>
+          <t>35663</t>
         </is>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>44 kg</t>
         </is>
       </c>
       <c r="O11" s="11" t="n">
@@ -1556,16 +1556,16 @@
         </is>
       </c>
       <c r="C22" s="11" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>35087</t>
+          <t>35080</t>
         </is>
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>45 kg</t>
         </is>
       </c>
       <c r="F22" s="11" t="n">
@@ -10713,7 +10713,7 @@
         <v>132</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="G9" s="14" t="n">
         <v>636</v>
@@ -10893,7 +10893,7 @@
         </is>
       </c>
       <c r="C18" s="14" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D18" s="14" t="n">
         <v>631</v>
@@ -13960,16 +13960,16 @@
         </is>
       </c>
       <c r="J7" s="18" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="K7" s="19" t="inlineStr">
         <is>
-          <t>35080</t>
+          <t>35663</t>
         </is>
       </c>
       <c r="L7" s="13" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>44 kg</t>
         </is>
       </c>
       <c r="M7" s="18" t="n">
@@ -14344,16 +14344,16 @@
     </row>
     <row r="13">
       <c r="A13" s="18" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="B13" s="19" t="inlineStr">
         <is>
-          <t>35087</t>
+          <t>35080</t>
         </is>
       </c>
       <c r="C13" s="13" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>45 kg</t>
         </is>
       </c>
       <c r="D13" s="18" t="n">
@@ -20527,7 +20527,7 @@
         <v>6</v>
       </c>
       <c r="I8" s="23" t="n">
-        <v>1455</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -20557,7 +20557,7 @@
         <v>6</v>
       </c>
       <c r="I9" s="25" t="n">
-        <v>1448</v>
+        <v>1459</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -21455,21 +21455,21 @@
         <v>10</v>
       </c>
       <c r="C38" s="31" t="n">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="D38" s="32" t="inlineStr">
         <is>
-          <t>35080</t>
+          <t>35663</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F38" s="33" t="inlineStr">
         <is>
-          <t>45 kg</t>
+          <t>44 kg</t>
         </is>
       </c>
       <c r="G38" s="30" t="inlineStr">
@@ -22616,11 +22616,11 @@
         <v>37</v>
       </c>
       <c r="C65" s="18" t="n">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>35087</t>
+          <t>35080</t>
         </is>
       </c>
       <c r="E65" s="28" t="inlineStr">
@@ -22630,7 +22630,7 @@
       </c>
       <c r="F65" s="29" t="inlineStr">
         <is>
-          <t>34 kg</t>
+          <t>45 kg</t>
         </is>
       </c>
       <c r="G65" s="28" t="inlineStr">

</xml_diff>